<commit_message>
Enforce campus scope; improve CSV import & UI
Add campus-aware access controls and improve bulk programme import and UI. Students API: refactor queries and add campusId enforcement in getStudentById/getStudents. Transcripts search now restricts results to session.campusId for non-SUPER_ADMIN. Bulk programmes CSV: stricter parsing/validation, flexible header names, composite (name+code) uniqueness, better error messages, and batch insert resilience. DB schema: add composite unique index on programmes (name, code). Misc: handle null campusId in JWT, UI tweaks to transcript preview/layout (add Vercel Analytics), remove setup link from login, update copy in programmes client, update templates and .gitignore.
</commit_message>
<xml_diff>
--- a/public/templates/courses-template.xlsx
+++ b/public/templates/courses-template.xlsx
@@ -46,6 +46,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00374151"/>
       <sz val="10"/>
     </font>
     <font>
@@ -148,9 +149,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,32 +515,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>credit_hours</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>is_scoring</t>
         </is>
@@ -558,11 +563,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -596,49 +601,49 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. course_code must be unique — duplicates will be automatically skipped.</t>
+          <t>3. The SAME course code can exist in different categories (e.g. UCC101 can be in</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>4. is_scoring: use 'true' for courses that count toward GPA, 'false' for others.</t>
+          <t xml:space="preserve">   OSIS_OLD and OSIS_NEW as two separate courses). Each code+category pair must be unique.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   If left blank, the course will be marked as scoring (true) by default.</t>
+          <t>4. is_scoring: use 'true' for GPA courses, 'false' for non-scoring (P/F) courses.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>5. credit_hours accepts any whole number — 2, 3, 6, 12, 18, 24 etc.</t>
+          <t xml:space="preserve">   Non-scoring courses only accept P (Pass) or F (Fail) as grades.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Save as CSV: File → Save As → CSV UTF-8 (Comma delimited) (*.csv)</t>
+          <t>5. Save as CSV: File → Save As → CSV UTF-8 (Comma delimited) (*.csv)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>7. Go to Bulk Upload → Course Import and upload the CSV file.</t>
+          <t>6. Go to Bulk Upload → Course Import and upload the CSV file.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>COLUMN REFERENCE</t>
+          <t>COURSE CATEGORIES</t>
         </is>
       </c>
     </row>
@@ -657,66 +662,146 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>OSIS_OLD</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Unique course code e.g. MATH101 — will be saved in UPPERCASE</t>
+          <t>Original OSIS courses (legacy — can still accept new grades)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>OSIS_NEW</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Full course title e.g. Introduction to Mathematics</t>
+          <t>New OSIS courses (current curriculum)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>credit_hours</t>
+          <t>ITS</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Number of credit hours — any value e.g. 2, 3, 6, 18, 24</t>
+          <t>ITS (Information Technology System) courses</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>OSIS_2</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>OSIS 2 courses (postgraduate / advanced level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>COLUMN REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Course category: OSIS_OLD, OSIS_NEW, ITS, or OSIS_2 (required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Course code — can repeat across categories e.g. MATH101 (required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Full course title (required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>credit_hours</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Number of credit hours — any whole number e.g. 2, 3, 6, 18, 24 (required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
           <t>is_scoring</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>true = counts toward GPA | false = non-scoring. Defaults to true if blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Example row: MATH101 | Introduction to Mathematics | 3 | true</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>true = counts toward GPA (standard grades A–F) | false = non-scoring (P/F only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Example: OSIS_NEW,MATH101,Introduction to Mathematics,3,true</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>

</xml_diff>